<commit_message>
docs: add more quantum diffusion literature
</commit_message>
<xml_diff>
--- a/metadata/Qdiffusion.xlsx
+++ b/metadata/Qdiffusion.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R284f3c2c0c3646a4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R74f09f060db043cc"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -614,19 +614,19 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="2" t="str">
-        <x:v>Mixed-state quantum denoising diffusion probabilistic model</x:v>
+        <x:v>Physics-inspired Generative AI models via real hardware-based noisy quantum diffusion</x:v>
       </x:c>
       <x:c r="B5" s="4" t="n">
-        <x:v>2025</x:v>
+        <x:v>2026</x:v>
       </x:c>
       <x:c r="C5" s="2" t="str">
-        <x:v>American Physical Society</x:v>
+        <x:v>Springer Nature</x:v>
       </x:c>
       <x:c r="D5" s="2" t="str">
-        <x:v>Gino Kwun; Bingzhi Zhang; Quntao Zhuang</x:v>
+        <x:v>Marco Parigi; Stefano Martina; Francesco Aldo Venturelli; Filippo Caruso</x:v>
       </x:c>
       <x:c r="E5" s="2" t="str">
-        <x:v>https://doi.org/10.1103/PhysRevA.111.032610</x:v>
+        <x:v>https://doi.org/10.1007/s42484-026-00459-5</x:v>
       </x:c>
       <x:c r="F5" s="2" t="str">
         <x:v>QDiffusion</x:v>
@@ -634,19 +634,19 @@
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="2" t="str">
-        <x:v>Quantum Diffusion Model for Quark and Gluon Jet Generation</x:v>
+        <x:v>Multimodal discrete diffusion for quantum measurement generation in the one-dimensional transverse-field Ising model</x:v>
       </x:c>
       <x:c r="B6" s="4" t="n">
-        <x:v>2025</x:v>
+        <x:v>2026</x:v>
       </x:c>
       <x:c r="C6" s="2" t="str">
-        <x:v>AAAI Symposium Series</x:v>
+        <x:v>American Physical Society</x:v>
       </x:c>
       <x:c r="D6" s="2" t="str">
-        <x:v>Mariia Baidachna; Rey Guadarrama; Gopal Ramesh Dahale; Tom Magorsch; Isabel Pedraza; Konstantin T. Matchev; Katia Matcheva; Kyoungchul Kong; Sergei Gleyzer</x:v>
+        <x:v>YanHong Li; Ho-Kin Tang</x:v>
       </x:c>
       <x:c r="E6" s="2" t="str">
-        <x:v>https://doi.org/10.1609/aaaiss.v7i1.36901</x:v>
+        <x:v>https://doi.org/10.1103/4tft-d7gf</x:v>
       </x:c>
       <x:c r="F6" s="2" t="str">
         <x:v>QDiffusion</x:v>
@@ -654,19 +654,19 @@
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="2" t="str">
-        <x:v>Quantum Diffusion Models for Few-Shot Learning</x:v>
+        <x:v>Mixed-state quantum denoising diffusion probabilistic model</x:v>
       </x:c>
       <x:c r="B7" s="4" t="n">
         <x:v>2025</x:v>
       </x:c>
       <x:c r="C7" s="2" t="str">
-        <x:v>IEEE</x:v>
+        <x:v>American Physical Society</x:v>
       </x:c>
       <x:c r="D7" s="2" t="str">
-        <x:v>Ruhan Wang; Ye Wang; Jing Liu; Toshiaki Koike-Akino</x:v>
+        <x:v>Gino Kwun; Bingzhi Zhang; Quntao Zhuang</x:v>
       </x:c>
       <x:c r="E7" s="2" t="str">
-        <x:v>https://doi.org/10.1109/ICAD65464.2025.11114033</x:v>
+        <x:v>https://doi.org/10.1103/PhysRevA.111.032610</x:v>
       </x:c>
       <x:c r="F7" s="2" t="str">
         <x:v>QDiffusion</x:v>
@@ -674,19 +674,19 @@
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="2" t="str">
-        <x:v>Denoising diffusion models with optimized quantum implicit neural networks for image generation</x:v>
+        <x:v>Quantum Diffusion Model for Quark and Gluon Jet Generation</x:v>
       </x:c>
       <x:c r="B8" s="4" t="n">
         <x:v>2025</x:v>
       </x:c>
       <x:c r="C8" s="2" t="str">
-        <x:v>Elsevier</x:v>
+        <x:v>AAAI Symposium Series</x:v>
       </x:c>
       <x:c r="D8" s="2" t="str">
-        <x:v>Jiale Zhang; Xilong Che; Yuzhe Fan; Shun Peng; Geng Chen; Quangong Ma; Juncheng Hu</x:v>
+        <x:v>Mariia Baidachna; Rey Guadarrama; Gopal Ramesh Dahale; Tom Magorsch; Isabel Pedraza; Konstantin T. Matchev; Katia Matcheva; Kyoungchul Kong; Sergei Gleyzer</x:v>
       </x:c>
       <x:c r="E8" s="2" t="str">
-        <x:v>https://doi.org/10.1016/j.future.2025.107875</x:v>
+        <x:v>https://doi.org/10.1609/aaaiss.v7i1.36901</x:v>
       </x:c>
       <x:c r="F8" s="2" t="str">
         <x:v>QDiffusion</x:v>
@@ -694,19 +694,19 @@
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="2" t="str">
-        <x:v>Quantum Latent Diffusion Models</x:v>
+        <x:v>Quantum Diffusion Models for Few-Shot Learning</x:v>
       </x:c>
       <x:c r="B9" s="4" t="n">
         <x:v>2025</x:v>
       </x:c>
       <x:c r="C9" s="2" t="str">
-        <x:v>arXiv</x:v>
+        <x:v>IEEE</x:v>
       </x:c>
       <x:c r="D9" s="2" t="str">
-        <x:v>Francesca De Falco; Andrea Ceschini; Alessandro Sebastianelli; Bertrand Le Saux; Massimo Panella</x:v>
+        <x:v>Ruhan Wang; Ye Wang; Jing Liu; Toshiaki Koike-Akino</x:v>
       </x:c>
       <x:c r="E9" s="2" t="str">
-        <x:v>https://arxiv.org/abs/2501.11174</x:v>
+        <x:v>https://doi.org/10.1109/ICAD65464.2025.11114033</x:v>
       </x:c>
       <x:c r="F9" s="2" t="str">
         <x:v>QDiffusion</x:v>
@@ -714,388 +714,388 @@
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="2" t="str">
+        <x:v>Denoising diffusion models with optimized quantum implicit neural networks for image generation</x:v>
+      </x:c>
+      <x:c r="B10" s="4" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="C10" s="2" t="str">
+        <x:v>Elsevier</x:v>
+      </x:c>
+      <x:c r="D10" s="2" t="str">
+        <x:v>Jiale Zhang; Xilong Che; Yuzhe Fan; Shun Peng; Geng Chen; Quangong Ma; Juncheng Hu</x:v>
+      </x:c>
+      <x:c r="E10" s="2" t="str">
+        <x:v>https://doi.org/10.1016/j.future.2025.107875</x:v>
+      </x:c>
+      <x:c r="F10" s="2" t="str">
+        <x:v>QDiffusion</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="2" t="str">
+        <x:v>Quantum Latent Diffusion Models</x:v>
+      </x:c>
+      <x:c r="B11" s="4" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="C11" s="2" t="str">
+        <x:v>arXiv</x:v>
+      </x:c>
+      <x:c r="D11" s="2" t="str">
+        <x:v>Francesca De Falco; Andrea Ceschini; Alessandro Sebastianelli; Bertrand Le Saux; Massimo Panella</x:v>
+      </x:c>
+      <x:c r="E11" t="str">
+        <x:v>https://arxiv.org/abs/2501.11174</x:v>
+      </x:c>
+      <x:c r="F11" s="2" t="str">
+        <x:v>QDiffusion</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="2" t="str">
+        <x:v>Quantum-Noise-Driven Generative Diffusion Models
+</x:v>
+      </x:c>
+      <x:c r="B12" s="4" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="C12" s="2" t="str">
+        <x:v>Advanced Quantum Technologies </x:v>
+      </x:c>
+      <x:c r="D12" s="2" t="str">
+        <x:v>Parigi, Marco, Stefano Martina, and Filippo Caruso.</x:v>
+      </x:c>
+      <x:c r="E12" s="2" t="str">
+        <x:v>https://onlinelibrary.wiley.com/doi/abs/10.1002/qute.202300401</x:v>
+      </x:c>
+      <x:c r="F12" s="2" t="str">
+        <x:v>QDiffusion</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="2" t="str">
+        <x:v>A Review of Quantum-Based Diffusion Models in Generative AI</x:v>
+      </x:c>
+      <x:c r="B13" s="4" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="C13" s="2" t="str">
+        <x:v>Vilnius University Open Series</x:v>
+      </x:c>
+      <x:c r="D13" s="2" t="str">
+        <x:v>Glauco Lima; Ernestas Filatovas; Marco Marcozzi; Remigijus Paulavičius</x:v>
+      </x:c>
+      <x:c r="E13" s="2" t="str">
+        <x:v>https://doi.org/10.15388/LMITT.2025.14</x:v>
+      </x:c>
+      <x:c r="F13" s="2" t="str">
+        <x:v>QDiffusion</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="2" t="str">
         <x:v>Quantum diffusion and large primordial perturbations from inflation
 </x:v>
       </x:c>
-      <x:c r="B10" s="4" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C10" s="2" t="str">
+      <x:c r="B14" s="4" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C14" s="2" t="str">
         <x:v>arXiv</x:v>
       </x:c>
-      <x:c r="D10" s="2" t="str">
+      <x:c r="D14" s="2" t="str">
         <x:v>Vennin, Vincent, and David Wands.</x:v>
       </x:c>
-      <x:c r="E10" s="2" t="str">
+      <x:c r="E14" s="2" t="str">
         <x:v>https://arxiv.org/abs/2402.12672</x:v>
       </x:c>
-      <x:c r="F10" s="2" t="str">
-        <x:v>QDiffusion</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="2" t="str">
+      <x:c r="F14" s="2" t="str">
+        <x:v>QDiffusion</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="2" t="str">
         <x:v>Asymptotic analysis of time-fractional quantum diffusion</x:v>
       </x:c>
-      <x:c r="B11" s="4" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C11" s="2" t="str">
+      <x:c r="B15" s="4" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C15" s="2" t="str">
         <x:v>Applied Mathematics Letters </x:v>
       </x:c>
-      <x:c r="D11" s="2" t="str">
+      <x:c r="D15" s="2" t="str">
         <x:v>Hislop, Peter D., and Eric Soccorsi.</x:v>
       </x:c>
-      <x:c r="E11" t="str">
+      <x:c r="E15" s="2" t="str">
         <x:v>https://www.sciencedirect.com/science/article/abs/pii/S0893965924000533</x:v>
       </x:c>
-      <x:c r="F11" s="2" t="str">
-        <x:v>QDiffusion</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12">
-      <x:c r="A12" s="2" t="str">
+      <x:c r="F15" s="2" t="str">
+        <x:v>QDiffusion</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="2" t="str">
         <x:v>Quantum Denoising Diffusion Models
 </x:v>
       </x:c>
-      <x:c r="B12" s="4" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C12" s="2" t="str">
+      <x:c r="B16" s="4" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C16" s="2" t="str">
         <x:v>arXiv</x:v>
       </x:c>
-      <x:c r="D12" s="2" t="str">
+      <x:c r="D16" s="2" t="str">
         <x:v>Kölle, Michael, et al.</x:v>
       </x:c>
-      <x:c r="E12" s="2" t="str">
+      <x:c r="E16" s="2" t="str">
         <x:v>https://arxiv.org/abs/2401.07049</x:v>
       </x:c>
-      <x:c r="F12" s="2" t="str">
-        <x:v>QDiffusion</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13">
-      <x:c r="A13" s="2" t="str">
+      <x:c r="F16" s="2" t="str">
+        <x:v>QDiffusion</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="2" t="str">
         <x:v>Corrections to Diffusion in Interacting Quantum Systems</x:v>
       </x:c>
-      <x:c r="B13" s="4" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C13" s="2" t="str">
+      <x:c r="B17" s="4" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C17" s="2" t="str">
         <x:v>Physical Review X </x:v>
       </x:c>
-      <x:c r="D13" s="2" t="str">
+      <x:c r="D17" s="2" t="str">
         <x:v>Michailidis, Alexios A., Dmitry A. Abanin, and Luca V. Delacrétaz.</x:v>
       </x:c>
-      <x:c r="E13" s="2" t="str">
+      <x:c r="E17" s="2" t="str">
         <x:v>https://journals.aps.org/prx/abstract/10.1103/PhysRevX.14.031020</x:v>
       </x:c>
-      <x:c r="F13" s="2" t="str">
-        <x:v>QDiffusion</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14">
-      <x:c r="A14" s="2" t="str">
+      <x:c r="F17" s="2" t="str">
+        <x:v>QDiffusion</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="2" t="str">
         <x:v>Generative quantum machine learning via denoising diffusion probabilistic models.</x:v>
       </x:c>
-      <x:c r="B14" s="4" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C14" s="2" t="str">
+      <x:c r="B18" s="4" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C18" s="2" t="str">
         <x:v>Physical Review Letters </x:v>
       </x:c>
-      <x:c r="D14" s="2" t="str">
+      <x:c r="D18" s="2" t="str">
         <x:v>Zhang, Bingzhi, et al.</x:v>
       </x:c>
-      <x:c r="E14" s="2" t="str">
+      <x:c r="E18" s="2" t="str">
         <x:v>https://journals.aps.org/prl/abstract/10.1103/PhysRevLett.132.100602</x:v>
       </x:c>
-      <x:c r="F14" s="2" t="str">
-        <x:v>QDiffusion</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15">
-      <x:c r="A15" s="2" t="str">
+      <x:c r="F18" s="2" t="str">
+        <x:v>QDiffusion</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="2" t="str">
         <x:v>Two quantum algorithms for solving the one-dimensional advection–diffusion equation</x:v>
       </x:c>
-      <x:c r="B15" s="4" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C15" s="2" t="str">
+      <x:c r="B19" s="4" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C19" s="2" t="str">
         <x:v>Computers &amp; Fluids</x:v>
       </x:c>
-      <x:c r="D15" s="2" t="str">
+      <x:c r="D19" s="2" t="str">
         <x:v>Ingelmann, Julia, et al.</x:v>
       </x:c>
-      <x:c r="E15" s="2" t="str">
+      <x:c r="E19" s="2" t="str">
         <x:v>https://www.sciencedirect.com/science/article/pii/S0045793024002019</x:v>
       </x:c>
-      <x:c r="F15" s="2" t="str">
-        <x:v>QDiffusion</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16">
-      <x:c r="A16" s="2" t="str">
+      <x:c r="F19" s="2" t="str">
+        <x:v>QDiffusion</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="2" t="str">
         <x:v>Clustering of primordial black holes from quantum diffusion during inflation
 </x:v>
       </x:c>
-      <x:c r="B16" s="4" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C16" s="2" t="str">
+      <x:c r="B20" s="4" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C20" s="2" t="str">
         <x:v>arXiv</x:v>
       </x:c>
-      <x:c r="D16" s="2" t="str">
+      <x:c r="D20" s="2" t="str">
         <x:v>Animali, Chiara, and Vincent Vennin.</x:v>
       </x:c>
-      <x:c r="E16" s="2" t="str">
+      <x:c r="E20" s="2" t="str">
         <x:v>https://arxiv.org/abs/2402.08642</x:v>
       </x:c>
-      <x:c r="F16" s="2" t="str">
-        <x:v>QDiffusion</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17">
-      <x:c r="A17" s="2" t="str">
+      <x:c r="F20" s="2" t="str">
+        <x:v>QDiffusion</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="2" t="str">
         <x:v>Quantum circuit synthesis with diffusion models
 </x:v>
       </x:c>
-      <x:c r="B17" s="4" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C17" s="2" t="str">
+      <x:c r="B21" s="4" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C21" s="2" t="str">
         <x:v>Nature Machine Intelligence </x:v>
       </x:c>
-      <x:c r="D17" s="2" t="str">
+      <x:c r="D21" s="2" t="str">
         <x:v>Fürrutter, Florian, Gorka Muñoz-Gil, and Hans J. Briegel.</x:v>
       </x:c>
-      <x:c r="E17" s="2" t="str">
+      <x:c r="E21" s="2" t="str">
         <x:v>https://www.nature.com/articles/s42256-024-00831-9</x:v>
       </x:c>
-      <x:c r="F17" s="2" t="str">
-        <x:v>QDiffusion</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18">
-      <x:c r="A18" s="2" t="str">
+      <x:c r="F21" s="2" t="str">
+        <x:v>QDiffusion</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="2" t="str">
         <x:v>Quantum State Generation with Structure-Preserving
 Diffusion Model</x:v>
       </x:c>
-      <x:c r="B18" s="4" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C18" s="2" t="str">
+      <x:c r="B22" s="4" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C22" s="2" t="str">
         <x:v>arXiv</x:v>
       </x:c>
-      <x:c r="D18" s="2" t="str">
+      <x:c r="D22" s="2" t="str">
         <x:v>Zhu, Yuchen, et al.</x:v>
       </x:c>
-      <x:c r="E18" s="2" t="str">
+      <x:c r="E22" s="2" t="str">
         <x:v>https://arxiv.org/abs/2404.06336</x:v>
       </x:c>
-      <x:c r="F18" s="2" t="str">
-        <x:v>QDiffusion</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="2" t="str">
+      <x:c r="F22" s="2" t="str">
+        <x:v>QDiffusion</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" s="3" customFormat="1">
+      <x:c r="A23" s="3" t="str">
         <x:v>variational Quantum Simulation of Lindblad Dynamics via Quantum State Diffusion</x:v>
       </x:c>
-      <x:c r="B19" s="4" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C19" s="2" t="str">
+      <x:c r="B23" s="5" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C23" s="3" t="str">
         <x:v>The Journal of Physical Chemistry Letters </x:v>
       </x:c>
-      <x:c r="D19" s="2" t="str">
+      <x:c r="D23" s="3" t="str">
         <x:v>Luo, Jianming, Kaihan Lin, and Xing Gao.</x:v>
       </x:c>
-      <x:c r="E19" s="2" t="str">
+      <x:c r="E23" s="3" t="str">
         <x:v>https://pubs.acs.org/doi/10.1021/acs.jpclett.4c00576</x:v>
       </x:c>
-      <x:c r="F19" s="2" t="str">
-        <x:v>QDiffusion</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20">
-      <x:c r="A20" s="2" t="str">
+      <x:c r="F23" s="3" t="str">
+        <x:v>QDiffusion</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" s="3" customFormat="1">
+      <x:c r="A24" s="3" t="str">
         <x:v>Quantum diffusion models for quantum data learning in
 high-energy physics</x:v>
       </x:c>
-      <x:c r="B20" s="4" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C20" s="2"/>
-      <x:c r="D20" s="2" t="str">
+      <x:c r="B24" s="5" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C24" s="3"/>
+      <x:c r="D24" s="3" t="str">
         <x:v>Cacioppo, Andrea, et al.</x:v>
       </x:c>
-      <x:c r="E20" s="2" t="str">
+      <x:c r="E24" s="3" t="str">
         <x:v>https://indico.qtml2024.org/event/1/contributions/178/attachments/178/183/QuantumDiffusion_forHEP_QTML2024.pdf</x:v>
       </x:c>
-      <x:c r="F20" s="2" t="str">
-        <x:v>QDiffusion</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="21">
-      <x:c r="A21" s="2" t="str">
+      <x:c r="F24" s="3" t="str">
+        <x:v>QDiffusion</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" s="3" customFormat="1">
+      <x:c r="A25" s="3" t="str">
         <x:v>Diffusion quantum Monte Carlo approach to the polaritonic ground state</x:v>
       </x:c>
-      <x:c r="B21" s="4" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C21" s="2" t="str">
+      <x:c r="B25" s="5" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C25" s="3" t="str">
         <x:v>Physical Review A</x:v>
       </x:c>
-      <x:c r="D21" s="2" t="str">
+      <x:c r="D25" s="3" t="str">
         <x:v>Weight, Braden M., Sergei Tretiak, and Yu Zhang.</x:v>
       </x:c>
-      <x:c r="E21" s="2" t="str">
+      <x:c r="E25" s="3" t="str">
         <x:v>https://journals.aps.org/pra/abstract/10.1103/PhysRevA.109.032804</x:v>
       </x:c>
-      <x:c r="F21" s="2" t="str">
-        <x:v>QDiffusion</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="22">
-      <x:c r="A22" s="2" t="str">
+      <x:c r="F25" s="3" t="str">
+        <x:v>QDiffusion</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="3" t="str">
         <x:v>Diffusion, Long-Time Tails, and Localization in Classical and Quantum Lorentz Models: A Unifying Hydrodynamic Approach
 </x:v>
       </x:c>
-      <x:c r="B22" s="4" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C22" s="2" t="str">
+      <x:c r="B26" s="5" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C26" s="3" t="str">
         <x:v>arXiv</x:v>
       </x:c>
-      <x:c r="D22" s="2" t="str">
+      <x:c r="D26" s="3" t="str">
         <x:v>Kirkpatrick, T. R., and D. Belitz.</x:v>
       </x:c>
-      <x:c r="E22" s="2" t="str">
+      <x:c r="E26" s="3" t="str">
         <x:v>https://arxiv.org/abs/2409.08123</x:v>
       </x:c>
-      <x:c r="F22" s="2" t="str">
-        <x:v>QDiffusion</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="23" s="3" customFormat="1">
-      <x:c r="A23" s="3" t="str">
-        <x:v>Quantum-Noise-Driven Generative Diffusion Models
-</x:v>
-      </x:c>
-      <x:c r="B23" s="5" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C23" s="3" t="str">
-        <x:v>Advanced Quantum Technologies </x:v>
-      </x:c>
-      <x:c r="D23" s="3" t="str">
-        <x:v>Parigi, Marco, Stefano Martina, and Filippo Caruso.</x:v>
-      </x:c>
-      <x:c r="E23" s="3" t="str">
-        <x:v>https://onlinelibrary.wiley.com/doi/abs/10.1002/qute.202300401</x:v>
-      </x:c>
-      <x:c r="F23" s="3" t="str">
-        <x:v>QDiffusion</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="24" s="3" customFormat="1">
-      <x:c r="A24" s="3" t="str">
+      <x:c r="F26" s="3" t="str">
+        <x:v>QDiffusion</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="3" t="str">
         <x:v>Quantum Generative Diffusion Model: A Fully
 Quantum-Mechanical Model for Generating
 Quantum State Ensemble</x:v>
       </x:c>
-      <x:c r="B24" s="5" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C24" s="3" t="str">
+      <x:c r="B27" s="5" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C27" s="3" t="str">
         <x:v>arXiv</x:v>
       </x:c>
-      <x:c r="D24" s="3" t="str">
+      <x:c r="D27" s="3" t="str">
         <x:v>vennin, Vincent, and David Wands.</x:v>
       </x:c>
-      <x:c r="E24" s="3" t="str">
+      <x:c r="E27" s="3" t="str">
         <x:v>https://arxiv.org/abs/2401.07039</x:v>
       </x:c>
-      <x:c r="F24" s="3" t="str">
-        <x:v>QDiffusion</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="25" s="3" customFormat="1">
-      <x:c r="A25" s="3" t="str">
+      <x:c r="F27" s="3" t="str">
+        <x:v>QDiffusion</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="3" t="str">
         <x:v>Towards Efficient Quantum Hybrid Diffusion Models
 </x:v>
       </x:c>
-      <x:c r="B25" s="5" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C25" s="3" t="str">
+      <x:c r="B28" s="5" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C28" s="3" t="str">
         <x:v>arXiv</x:v>
       </x:c>
-      <x:c r="D25" s="3" t="str">
+      <x:c r="D28" s="3" t="str">
         <x:v>De Falco, Francesca, et al.</x:v>
       </x:c>
-      <x:c r="E25" s="3" t="str">
+      <x:c r="E28" s="3" t="str">
         <x:v>https://arxiv.org/pdf/2402.16147</x:v>
-      </x:c>
-      <x:c r="F25" s="3" t="str">
-        <x:v>QDiffusion</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="26">
-      <x:c r="A26" s="3" t="str">
-        <x:v>Quantum diffusion in sharp transition to non-slow-roll phase</x:v>
-      </x:c>
-      <x:c r="B26" s="5" t="n">
-        <x:v>2022</x:v>
-      </x:c>
-      <x:c r="C26" s="3" t="str">
-        <x:v>Journal of Cosmology and Astroparticle Physics</x:v>
-      </x:c>
-      <x:c r="D26" s="3" t="str">
-        <x:v>Nahid Ahmadi1, Mahdiyar Noorbala1,2, Niloufar Feyzabadi1, Fatemeh Eghbalpoor1 and Zahra Ahmadi</x:v>
-      </x:c>
-      <x:c r="E26" s="3" t="str">
-        <x:v>https://iopscience.iop.org/article/10.1088/1475-7516/2022/08/078/meta</x:v>
-      </x:c>
-      <x:c r="F26" s="3" t="str">
-        <x:v>QDiffusion</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="27">
-      <x:c r="A27" s="3" t="str">
-        <x:v>Variational quantum solutions to the advection–diffusion equation for applications in fluid dynamics</x:v>
-      </x:c>
-      <x:c r="B27" s="5" t="n">
-        <x:v>2022</x:v>
-      </x:c>
-      <x:c r="C27" s="3" t="str">
-        <x:v>Quantum Information Processing</x:v>
-      </x:c>
-      <x:c r="D27" s="3" t="str">
-        <x:v>      Reuben Demirdjian, Daniel Gunlycke, …Sergio Tafur   </x:v>
-      </x:c>
-      <x:c r="E27" s="3" t="str">
-        <x:v>https://link.springer.com/article/10.1007/s11128-022-03667-7</x:v>
-      </x:c>
-      <x:c r="F27" s="3" t="str">
-        <x:v>QDiffusion</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="28">
-      <x:c r="A28" s="3" t="str">
-        <x:v>Learning Quantum Drift-Diffusion Phenomenon by Physics-Constraint Machine Learning</x:v>
-      </x:c>
-      <x:c r="B28" s="5" t="n">
-        <x:v>2022</x:v>
-      </x:c>
-      <x:c r="C28" s="3" t="str">
-        <x:v>IEEE/ACM Transactions </x:v>
-      </x:c>
-      <x:c r="D28" s="3" t="str">
-        <x:v>Chun Li School of Science, Harbin Institute of Technology, Shenzhen, China ; Yunyun Yang; Hui Liang; Boying Wu</x:v>
-      </x:c>
-      <x:c r="E28" s="3" t="str">
-        <x:v>https://ieeexplore.ieee.org/abstract/document/9751143</x:v>
       </x:c>
       <x:c r="F28" s="3" t="str">
         <x:v>QDiffusion</x:v>
@@ -1103,19 +1103,19 @@
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="3" t="str">
-        <x:v>Many-Body Quantum State Diffusion for Non-Markovian Dynamics in Strongly Interacting Systems</x:v>
+        <x:v>Quantum diffusion in sharp transition to non-slow-roll phase</x:v>
       </x:c>
       <x:c r="B29" s="5" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C29" s="3" t="str">
-        <x:v>Phys. Rev. Lett. 128</x:v>
+        <x:v>Journal of Cosmology and Astroparticle Physics</x:v>
       </x:c>
       <x:c r="D29" s="3" t="str">
-        <x:v>S. Flannigan, F. Damanet, and A. J. Daley</x:v>
+        <x:v>Nahid Ahmadi1, Mahdiyar Noorbala1,2, Niloufar Feyzabadi1, Fatemeh Eghbalpoor1 and Zahra Ahmadi</x:v>
       </x:c>
       <x:c r="E29" s="3" t="str">
-        <x:v>https://journals.aps.org/prl/abstract/10.1103/PhysRevLett.128.063601</x:v>
+        <x:v>https://iopscience.iop.org/article/10.1088/1475-7516/2022/08/078/meta</x:v>
       </x:c>
       <x:c r="F29" s="3" t="str">
         <x:v>QDiffusion</x:v>
@@ -1123,19 +1123,19 @@
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="3" t="str">
-        <x:v>Research on Quantum Communication Technology Based on Markov's Quantum Diffusion</x:v>
+        <x:v>Variational quantum solutions to the advection–diffusion equation for applications in fluid dynamics</x:v>
       </x:c>
       <x:c r="B30" s="5" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C30" s="3" t="str">
-        <x:v>2022 2nd International Signal Processing, Communications and Engineering Management Conference (ISPCEM)</x:v>
+        <x:v>Quantum Information Processing</x:v>
       </x:c>
       <x:c r="D30" s="3" t="str">
-        <x:v>Wenyu Hu; Min Nie</x:v>
+        <x:v>      Reuben Demirdjian, Daniel Gunlycke, …Sergio Tafur   </x:v>
       </x:c>
       <x:c r="E30" s="3" t="str">
-        <x:v>https://ieeexplore.ieee.org/abstract/document/10070269</x:v>
+        <x:v>https://link.springer.com/article/10.1007/s11128-022-03667-7</x:v>
       </x:c>
       <x:c r="F30" s="3" t="str">
         <x:v>QDiffusion</x:v>
@@ -1143,19 +1143,19 @@
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="3" t="str">
-        <x:v>Diffusion Monte Carlo approaches for studying nuclear quantum effects in fluxional molecules</x:v>
+        <x:v>Learning Quantum Drift-Diffusion Phenomenon by Physics-Constraint Machine Learning</x:v>
       </x:c>
       <x:c r="B31" s="5" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C31" s="3" t="str">
-        <x:v>WIREs Computational Molecular Science</x:v>
+        <x:v>IEEE/ACM Transactions </x:v>
       </x:c>
       <x:c r="D31" s="3" t="str">
-        <x:v>Ryan J. DiRisio, Jacob M. Finney, Anne B. McCoy</x:v>
+        <x:v>Chun Li School of Science, Harbin Institute of Technology, Shenzhen, China ; Yunyun Yang; Hui Liang; Boying Wu</x:v>
       </x:c>
       <x:c r="E31" s="3" t="str">
-        <x:v>https://wires.onlinelibrary.wiley.com/doi/abs/10.1002/wcms.1615</x:v>
+        <x:v>https://ieeexplore.ieee.org/abstract/document/9751143</x:v>
       </x:c>
       <x:c r="F31" s="3" t="str">
         <x:v>QDiffusion</x:v>
@@ -1163,19 +1163,19 @@
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="3" t="str">
-        <x:v>Diffusion Quantum-Least Mean Square Algorithm with Steady-State Analysis</x:v>
+        <x:v>Many-Body Quantum State Diffusion for Non-Markovian Dynamics in Strongly Interacting Systems</x:v>
       </x:c>
       <x:c r="B32" s="5" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C32" s="3" t="str">
-        <x:v>Circuits, Systems, and Signal Processing</x:v>
+        <x:v>Phys. Rev. Lett. 128</x:v>
       </x:c>
       <x:c r="D32" s="3" t="str">
-        <x:v>    Muhammad Arif, Muhammad Moinuddin, Imran Naseem, Abdulrahman U. Alsaggaf &amp; Ubaid M. Al-Saggaf </x:v>
+        <x:v>S. Flannigan, F. Damanet, and A. J. Daley</x:v>
       </x:c>
       <x:c r="E32" s="3" t="str">
-        <x:v>https://link.springer.com/article/10.1007/s00034-021-01934-z</x:v>
+        <x:v>https://journals.aps.org/prl/abstract/10.1103/PhysRevLett.128.063601</x:v>
       </x:c>
       <x:c r="F32" s="3" t="str">
         <x:v>QDiffusion</x:v>
@@ -1183,30 +1183,90 @@
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="3" t="str">
-        <x:v>Modeling quantum diffusion in linear aggregates coupled to colored noise baths</x:v>
+        <x:v>Research on Quantum Communication Technology Based on Markov's Quantum Diffusion</x:v>
       </x:c>
       <x:c r="B33" s="5" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C33" s="3" t="str">
+        <x:v>2022 2nd International Signal Processing, Communications and Engineering Management Conference (ISPCEM)</x:v>
+      </x:c>
+      <x:c r="D33" s="3" t="str">
+        <x:v>Wenyu Hu; Min Nie</x:v>
+      </x:c>
+      <x:c r="E33" s="3" t="str">
+        <x:v>https://ieeexplore.ieee.org/abstract/document/10070269</x:v>
+      </x:c>
+      <x:c r="F33" s="3" t="str">
+        <x:v>QDiffusion</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="3" t="str">
+        <x:v>Diffusion Monte Carlo approaches for studying nuclear quantum effects in fluxional molecules</x:v>
+      </x:c>
+      <x:c r="B34" s="5" t="n">
+        <x:v>2022</x:v>
+      </x:c>
+      <x:c r="C34" s="3" t="str">
+        <x:v>WIREs Computational Molecular Science</x:v>
+      </x:c>
+      <x:c r="D34" s="3" t="str">
+        <x:v>Ryan J. DiRisio, Jacob M. Finney, Anne B. McCoy</x:v>
+      </x:c>
+      <x:c r="E34" s="3" t="str">
+        <x:v>https://wires.onlinelibrary.wiley.com/doi/abs/10.1002/wcms.1615</x:v>
+      </x:c>
+      <x:c r="F34" s="3" t="str">
+        <x:v>QDiffusion</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" s="3" t="str">
+        <x:v>Diffusion Quantum-Least Mean Square Algorithm with Steady-State Analysis</x:v>
+      </x:c>
+      <x:c r="B35" s="5" t="n">
+        <x:v>2022</x:v>
+      </x:c>
+      <x:c r="C35" s="3" t="str">
+        <x:v>Circuits, Systems, and Signal Processing</x:v>
+      </x:c>
+      <x:c r="D35" s="3" t="str">
+        <x:v>    Muhammad Arif, Muhammad Moinuddin, Imran Naseem, Abdulrahman U. Alsaggaf &amp; Ubaid M. Al-Saggaf </x:v>
+      </x:c>
+      <x:c r="E35" s="3" t="str">
+        <x:v>https://link.springer.com/article/10.1007/s00034-021-01934-z</x:v>
+      </x:c>
+      <x:c r="F35" s="3" t="str">
+        <x:v>QDiffusion</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" s="3" t="str">
+        <x:v>Modeling quantum diffusion in linear aggregates coupled to colored noise baths</x:v>
+      </x:c>
+      <x:c r="B36" s="5" t="n">
+        <x:v>2022</x:v>
+      </x:c>
+      <x:c r="C36" s="3" t="str">
         <x:v>Bachelor's Thesis, Physics.</x:v>
       </x:c>
-      <x:c r="D33" s="3" t="str">
+      <x:c r="D36" s="3" t="str">
         <x:v>Wobben, Hans Douwe</x:v>
       </x:c>
-      <x:c r="E33" s="3" t="str">
+      <x:c r="E36" s="3" t="str">
         <x:v>https://fse.studenttheses.ub.rug.nl/27743/</x:v>
       </x:c>
-      <x:c r="F33" s="3" t="str">
+      <x:c r="F36" s="3" t="str">
         <x:v>QDiffusion</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="Rfc6f431cab0a43df"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="Re6238e5500ea472d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="R15717f8f8e594e0a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="R8921305933a3444b"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra5bbc0b504e24430"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfa34a96314b3498f"/>
 </x:worksheet>
 </file>
</xml_diff>